<commit_message>
added all active user
</commit_message>
<xml_diff>
--- a/src/test/resources/Team01_RestAssured_Rebels_TestDataSheet.xlsx
+++ b/src/test/resources/Team01_RestAssured_Rebels_TestDataSheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dineshdeshmukh/eclipse-workspace/Team01_RestAssured_Rebels/src/test/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2822732F-7638-4B46-951F-FB0ABF6696EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07BAE372-DE15-194A-8D0D-747CE914152B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="1300" windowWidth="38400" windowHeight="18900" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38400" yWindow="1300" windowWidth="38400" windowHeight="18800" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="60">
   <si>
     <t>ScenarioName</t>
   </si>
@@ -146,33 +146,6 @@
   "userRoleMaps": [
     {
       "roleId": "R02",
-      "userRoleStatus": "Active"
-    }
-  ],
-  "userLogin": {
-    "userLoginEmail": "&lt;random_email&gt;",
-    "loginStatus": "Active",
-    "status": "Active"
-  }
-}</t>
-  </si>
-  <si>
-    <t>{
-  "userFirstName": "sunny",
-  "userLastName": "penny",
-  "userMiddleName": "jonn",
-  "userPhoneNumber": "&lt;random_phone&gt;",
-  "userEmail": "&lt;random_email&gt;",
-  "userLocation": "Atlanta",
-  "userTimeZone": "EST",
-  "userLinkedinUrl": "www.linkedin.com",
-  "userEduUg": "BE",
-  "userEduPg": "PHD",
-  "userComments": "PASSED",
-  "userVisaStatus": "H1B",
-  "userRoleMaps": [
-    {
-      "roleId": "R03",
       "userRoleStatus": "Active"
     }
   ],
@@ -424,27 +397,6 @@
     <t>Create_User_Empty_LoginStatus</t>
   </si>
   <si>
-    <t>{
-  "userFirstName": "Sunny",
-  "userLastName": "Penny",
-  "userPhoneNumber": "&lt;random_phone&gt;",
-  "userLocation": "Atlanta",
-  "userTimeZone": "EST",
-  "userVisaStatus": "H4",
-  "userRoleMaps": [
-    {
-      "roleId": "R03",
-      "userRoleStatus": "Active"
-    }
-  ],
-  "userLogin": {
-    "userLoginEmail": "&lt;random_email&gt;",
-    "loginStatus": "",
-    "status": "Active"
-  }
-}</t>
-  </si>
-  <si>
     <t xml:space="preserve">Create_User_Empty_Email </t>
   </si>
   <si>
@@ -494,6 +446,77 @@
   </si>
   <si>
     <t>Create_User_Only_Mandatory_Field</t>
+  </si>
+  <si>
+    <t>Get_All_Active_Users_Success</t>
+  </si>
+  <si>
+    <t>/users/activeUsers</t>
+  </si>
+  <si>
+    <t>Get_All_Active_Users_Invalid_Endpoint</t>
+  </si>
+  <si>
+    <t>Get_All_Active_Users_Invalid_Method</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Get_All_Active_Users_No_Auth </t>
+  </si>
+  <si>
+    <t>/use/activeUsers</t>
+  </si>
+  <si>
+    <t>Auth</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "sunny",
+  "userLastName": "penny",
+  "userMiddleName": "jonn",
+  "userPhoneNumber": "&lt;random_phone&gt;",
+    "userLocation": "Atlanta",
+  "userTimeZone": "EST",
+  "userLinkedinUrl": "www.linkedin.com",
+  "userEduUg": "BE",
+  "userEduPg": "PHD",
+  "userComments": "PASSED",
+  "userVisaStatus": "H1B",
+  "userRoleMaps": [
+    {
+      "roleId": "R03",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "Sunny",
+  "userLastName": "Penny",
+  "userPhoneNumber": "&lt;random_phone&gt;",
+  "userLocation": "Atlanta",
+  "userTimeZone": "EST",
+  "userVisaStatus": "H4",
+  "userRoleMaps": [
+    {
+      "roleId": "R03",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": " ",
+    "status": "Active"
+  }
+}</t>
   </si>
 </sst>
 </file>
@@ -10144,7 +10167,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5ECCC9A2-780E-422B-AA2C-B36256EC8A5E}">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.83203125" style="11"/>
@@ -10152,7 +10175,7 @@
     <col min="3" max="16384" width="8.83203125" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="29" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="29" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -10165,8 +10188,14 @@
       <c r="D1" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="333" x14ac:dyDescent="0.2">
+      <c r="E1" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="333" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>21</v>
       </c>
@@ -10180,12 +10209,12 @@
         <v>201</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="395" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" ht="380" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>22</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>26</v>
+        <v>58</v>
       </c>
       <c r="C3" s="11" t="s">
         <v>20</v>
@@ -10194,12 +10223,12 @@
         <v>201</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="380" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" ht="380" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>23</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>20</v>
@@ -10208,12 +10237,12 @@
         <v>201</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" ht="304" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>24</v>
@@ -10222,12 +10251,12 @@
         <v>201</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="64" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" ht="64" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="11" t="s">
         <v>29</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>30</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>24</v>
@@ -10236,12 +10265,12 @@
         <v>400</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="380" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" ht="380" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="11" t="s">
         <v>31</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>32</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>24</v>
@@ -10250,12 +10279,12 @@
         <v>400</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="380" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" ht="380" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>24</v>
@@ -10264,12 +10293,12 @@
         <v>400</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="380" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" ht="380" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>24</v>
@@ -10278,12 +10307,12 @@
         <v>400</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" ht="304" x14ac:dyDescent="0.2">
       <c r="A10" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>24</v>
@@ -10292,12 +10321,12 @@
         <v>400</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" ht="304" x14ac:dyDescent="0.2">
       <c r="A11" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" s="11" t="s">
         <v>39</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>40</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>24</v>
@@ -10306,12 +10335,12 @@
         <v>400</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" ht="304" x14ac:dyDescent="0.2">
       <c r="A12" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" s="11" t="s">
         <v>41</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>42</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>24</v>
@@ -10320,12 +10349,12 @@
         <v>400</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" ht="304" x14ac:dyDescent="0.2">
       <c r="A13" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" s="11" t="s">
         <v>43</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>44</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>24</v>
@@ -10334,12 +10363,12 @@
         <v>400</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" ht="304" x14ac:dyDescent="0.2">
       <c r="A14" s="11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>24</v>
@@ -10348,12 +10377,12 @@
         <v>400</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" ht="304" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>24</v>
@@ -10362,18 +10391,77 @@
         <v>400</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" ht="304" x14ac:dyDescent="0.2">
       <c r="A16" s="11" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C16" s="11" t="s">
         <v>24</v>
       </c>
       <c r="D16" s="11">
         <v>400</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+      <c r="A17" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="D17" s="11">
+        <v>200</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="80" x14ac:dyDescent="0.2">
+      <c r="A18" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="D18" s="11">
+        <v>404</v>
+      </c>
+      <c r="E18" s="11" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+      <c r="A19" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="D19" s="11">
+        <v>405</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+      <c r="A20" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="D20" s="11">
+        <v>401</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added Active email users
</commit_message>
<xml_diff>
--- a/src/test/resources/Team01_RestAssured_Rebels_TestDataSheet.xlsx
+++ b/src/test/resources/Team01_RestAssured_Rebels_TestDataSheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dineshdeshmukh/eclipse-workspace/Team01_RestAssured_Rebels/src/test/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EB3BF46-7AC1-1A47-8564-0F44CB17DCCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04C7E07E-20C8-BB4E-A370-02CDC98C9688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="1560" windowWidth="38400" windowHeight="18800" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38240" yWindow="1460" windowWidth="38080" windowHeight="17780" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="106">
   <si>
     <t>ScenarioName</t>
   </si>
@@ -129,32 +129,6 @@
   </si>
   <si>
     <t>/users/roleStatus</t>
-  </si>
-  <si>
-    <t>{
-  "userFirstName": "Pamm",
-  "userLastName": "Dasd",
-  "userMiddleName": "Pdn",
-  "userPhoneNumber": "&lt;random_phone&gt;",
-  "userLocation": "Atlanta",
-  "userTimeZone": "EST",
-  "userLinkedinUrl": "www.linkedin.com",
-  "userEduUg": "BE",
-  "userEduPg": "PHD",
-  "userComments": "PASSED",
-  "userVisaStatus": "H1B",
-  "userRoleMaps": [
-    {
-      "roleId": "R02",
-      "userRoleStatus": "Active"
-    }
-  ],
-  "userLogin": {
-    "userLoginEmail": "&lt;random_email&gt;",
-    "loginStatus": "Active",
-    "status": "Active"
-  }
-}</t>
   </si>
   <si>
     <t>{
@@ -296,27 +270,6 @@
   </si>
   <si>
     <t>Create_User_Empty_Location</t>
-  </si>
-  <si>
-    <t>{
-  "userFirstName": "Sunny",
-  "userLastName": "Penny",
-  "userPhoneNumber": "&lt;random_phone&gt;",
-  "userLocation": "Atlanta",
-  "userTimeZone": "",
-  "userVisaStatus": "H1B",
-  "userRoleMaps": [
-    {
-      "roleId": "R01",
-      "userRoleStatus": "Active"
-    }
-  ],
-  "userLogin": {
-    "userLoginEmail": "&lt;random_email&gt;",
-    "loginStatus": "Active",
-    "status": "Active"
-  }
-}</t>
   </si>
   <si>
     <t>Create_User_Empty_TimeZone</t>
@@ -518,12 +471,532 @@
   }
 }</t>
   </si>
+  <si>
+    <t>Get_Active_User_Emails_Valid_Endpoint</t>
+  </si>
+  <si>
+    <t>Get_Active_User_Emails_Invalid_Method</t>
+  </si>
+  <si>
+    <t>Get_Active_User_Emails_No_Auth</t>
+  </si>
+  <si>
+    <t>/fetch-emails</t>
+  </si>
+  <si>
+    <t>GET</t>
+  </si>
+  <si>
+    <t>/fetch-Invalidemailseeeee</t>
+  </si>
+  <si>
+    <t>Get_Active_User_Emails_Invalid_Endpoint</t>
+  </si>
+  <si>
+    <t>Create_User_Duplicate_Email</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "Sunny",
+  "userLastName": "Penny","userMiddleName": "Desi",
+  "userPhoneNumber": "&lt;random_phone&gt;",
+  "userLocation": "Atlanta",
+  "userTimeZone": "",
+  "userVisaStatus": "H1B",
+  "userRoleMaps": [
+    {
+      "roleId": "R01",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "Sunny",
+  "userLastName": "Penny","userMiddleName": "Desi",
+  "userPhoneNumber": "&lt;random_phone&gt;",
+  "userLocation": "Atlanta",
+  "userTimeZone": "EST",
+  "userVisaStatus": "H1B",
+  "userRoleMaps": [
+    {
+      "roleId": "R01",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "Team01@gmail.com",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t>Create_User_Duplicate_Phone_Number</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "Sunny",
+  "userLastName": "Penny",
+  "userPhoneNumber": "+91 9158758687",
+  "userLocation": "Atlanta",
+  "userTimeZone": "EST",
+  "userVisaStatus": "H1B",
+  "userRoleMaps": [
+    {
+      "roleId": "R01",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t>Create_User_Invalid_UserEduPg</t>
+  </si>
+  <si>
+    <t>Create_User_Invalid_UserEduUg</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "Sunny",
+  "userLastName": "Patil",
+  "userMiddleName": "Desi",
+  "userPhoneNumber": "&lt;random_phone&gt;",
+  "userLocation": "Atlanta",
+  "userTimeZone": "EST",
+  "userLinkedinUrl": "www.linkedin.com",
+  "userEduUg": "123",
+  "userEduPg": "PHD",
+  "userComments": "PASSED",
+  "userVisaStatus": "H1B",
+  "userRoleMaps": [
+    {
+      "roleId": "R02",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "Sunny",
+  "userLastName": "Patil",
+  "userMiddleName": "Desi",
+  "userPhoneNumber": "&lt;random_phone&gt;",
+  "userLocation": "Atlanta",
+  "userTimeZone": "EST",
+  "userLinkedinUrl": "www.linkedin.com",
+  "userEduUg": "BE",
+  "userEduPg": "12356",
+  "userComments": "PASSED",
+  "userVisaStatus": "H1B",
+  "userRoleMaps": [
+    {
+      "roleId": "R02",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t>Create_User_Invalid_Last_Name</t>
+  </si>
+  <si>
+    <t>Create_User_Invalid_Middle_Name</t>
+  </si>
+  <si>
+    <t>Create_User_Invalid_UserLinkedinUrl</t>
+  </si>
+  <si>
+    <t>Create_User_Invalid_UserLocation</t>
+  </si>
+  <si>
+    <t>Create_User_Invalid_First_Name</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "123",
+  "userLastName": "Patil",
+  "userMiddleName": "Desi",
+  "userPhoneNumber": "&lt;random_phone&gt;",
+  "userLocation": "Atlanta",
+  "userTimeZone": "EST",
+  "userLinkedinUrl": "www.linkedin.com",
+  "userEduUg": "BE",
+  "userEduPg": "phd",
+  "userComments": "PASSED",
+  "userVisaStatus": "H1B",
+  "userRoleMaps": [
+    {
+      "roleId": "R02",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "Saloni",
+  "userLastName": "123",
+  "userMiddleName": "Desi",
+  "userPhoneNumber": "&lt;random_phone&gt;",
+  "userLocation": "Atlanta",
+  "userTimeZone": "EST",
+  "userLinkedinUrl": "www.linkedin.com",
+  "userEduUg": "BE",
+  "userEduPg": "phd",
+  "userComments": "PASSED",
+  "userVisaStatus": "H1B",
+  "userRoleMaps": [
+    {
+      "roleId": "R02",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "Saloni",
+  "userLastName": "Dubey",
+  "userMiddleName": "123",
+  "userPhoneNumber": "&lt;random_phone&gt;",
+  "userLocation": "Atlanta",
+  "userTimeZone": "EST",
+  "userLinkedinUrl": "www.linkedin.com",
+  "userEduUg": "BE",
+  "userEduPg": "Phd",
+  "userComments": "PASSED",
+  "userVisaStatus": "H1B",
+  "userRoleMaps": [
+    {
+      "roleId": "R02",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "Saloni",
+  "userLastName": "Dubey",
+  "userMiddleName": "das",
+  "userPhoneNumber": "&lt;random_phone&gt;",
+  "userLocation": "Atlanta",
+  "userTimeZone": "EST",
+  "userLinkedinUrl": "www.linkedinnnnn.in",
+  "userEduUg": "BE",
+  "userEduPg": "PHD",
+  "userComments": "PASSED",
+  "userVisaStatus": "H1B",
+  "userRoleMaps": [
+    {
+      "roleId": "R02",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "Saloni",
+  "userLastName": "Dubey",
+  "userMiddleName": "das",
+  "userPhoneNumber": "&lt;random_phone&gt;",
+  "userLocation": "123",
+  "userTimeZone": "EST",
+  "userLinkedinUrl": "www.linkedin.com",
+  "userEduUg": "BE",
+  "userEduPg": "PHD",
+  "userComments": "PASSED",
+  "userVisaStatus": "H1B",
+  "userRoleMaps": [
+    {
+      "roleId": "R02",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t>Create_User_Invalid_Phone_Number_Format</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "Saloni",
+  "userLastName": "Dubey",
+  "userMiddleName": "das",
+  "userPhoneNumber": " 5647839212. +91",
+  "userLocation": "India",
+  "userTimeZone": "EST",
+  "userLinkedinUrl": "www.linkedin.com",
+  "userEduUg": "BE",
+  "userEduPg": "PHD",
+  "userComments": "PASSED",
+  "userVisaStatus": "H1B",
+  "userRoleMaps": [
+    {
+      "roleId": "R02",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t>Create_User_Invalid_User_Role_Id</t>
+  </si>
+  <si>
+    <t>Create_User_Invalid_User_Role_Status</t>
+  </si>
+  <si>
+    <t>Create_User_Invalid_User_Time_Zone</t>
+  </si>
+  <si>
+    <t>Create_User_Invalid_User_Visa_Status</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "Saloni",
+  "userLastName": "Dubey",
+  "userMiddleName": "das",
+  "userPhoneNumber": "&lt;random_phone&gt;",
+  "userLocation": "India",
+  "userTimeZone": "EST",
+  "userLinkedinUrl": "www.linkedin.com",
+  "userEduUg": "BE",
+  "userEduPg": "PHD",
+  "userComments": "PASSED",
+  "userVisaStatus": "H1B",
+  "userRoleMaps": [
+    {
+      "roleId": "R03",
+      "userRoleStatus": "Present"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "Saloni",
+  "userLastName": "Dubey",
+  "userMiddleName": "das",
+  "userPhoneNumber": "&lt;random_phone&gt;",
+  "userLocation": "123",
+  "userTimeZone": "EST",
+  "userLinkedinUrl": "www.linkedin.com",
+  "userEduUg": "BE",
+  "userEduPg": "PHD",
+  "userComments": "PASSED",
+  "userVisaStatus": "H1B",
+  "userRoleMaps": [
+    {
+      "roleId": "R2",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "Saloni",
+  "userLastName": "Dubey",
+  "userMiddleName": "das",
+  "userPhoneNumber": "&lt;random_phone&gt;",
+  "userLocation": "India",
+  "userTimeZone": "PT",
+  "userLinkedinUrl": "www.linkedin.com",
+  "userEduUg": "BE",
+  "userEduPg": "PHD",
+  "userComments": "PASSED",
+  "userVisaStatus": "H1B",
+  "userRoleMaps": [
+    {
+      "roleId": "R03",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "Saloni",
+  "userLastName": "Dubey",
+  "userMiddleName": "das",
+  "userPhoneNumber": "&lt;random_phone&gt;",
+  "userLocation": "India",
+  "userTimeZone": "IST",
+  "userLinkedinUrl": "www.linkedin.com",
+  "userEduUg": "BE",
+  "userEduPg": "PHD",
+  "userComments": "PASSED",
+  "userVisaStatus": "NONE",
+  "userRoleMaps": [
+    {
+      "roleId": "R03",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t>Create_User_Invalid_Token</t>
+  </si>
+  <si>
+    <t>Create_User_Invalid_Endpoint</t>
+  </si>
+  <si>
+    <t>Create_User_Invalid_Content_Type</t>
+  </si>
+  <si>
+    <t>Create_User_Invalid_Method</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "Saloni",
+  "userLastName": "Dubey",
+  "userMiddleName": "das",
+  "userPhoneNumber": "&lt;random_phone&gt;",
+  "userLocation": "India",
+  "userTimeZone": "IST",
+  "userLinkedinUrl": "www.linkedin.com",
+  "userEduUg": "BE",
+  "userEduPg": "PHD",
+  "userComments": "PASSED",
+  "userVisaStatus": "NA",
+  "userRoleMaps": [
+    {
+      "roleId": "R03",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t>/api/v1/invalidpath123</t>
+  </si>
+  <si>
+    <t>ContentType</t>
+  </si>
+  <si>
+    <t>text/plain</t>
+  </si>
+  <si>
+    <t>PATCH</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "Neha",
+  "userLastName": "Patel",
+  "userMiddleName": "Das",
+  "userPhoneNumber": "&lt;random_phone&gt;",
+  "userLocation": "Atlanta",
+  "userTimeZone": "EST",
+  "userLinkedinUrl": "www.linkedin.com",
+  "userEduUg": "BE",
+  "userEduPg": "PHD",
+  "userComments": "PASSED",
+  "userVisaStatus": "H1B",
+  "userRoleMaps": [
+    {
+      "roleId": "R02",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t>application/json</t>
+  </si>
+  <si>
+    <t>Create_User_No_Auth</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -556,6 +1029,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -577,7 +1057,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -606,7 +1086,13 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -10167,54 +10653,69 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5ECCC9A2-780E-422B-AA2C-B36256EC8A5E}">
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.83203125" style="11"/>
+    <col min="1" max="1" width="31.6640625" style="11" customWidth="1"/>
     <col min="2" max="2" width="61.1640625" style="11" customWidth="1"/>
-    <col min="3" max="16384" width="8.83203125" style="11"/>
+    <col min="3" max="3" width="22.33203125" style="11" customWidth="1"/>
+    <col min="4" max="6" width="8.83203125" style="11"/>
+    <col min="7" max="7" width="23" style="11" customWidth="1"/>
+    <col min="8" max="16384" width="8.83203125" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="29" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="8" t="s">
         <v>19</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F1" s="11" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="333" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+      <c r="G1" s="11" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="332" x14ac:dyDescent="0.2">
+      <c r="A2" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C2" s="2" t="s">
+      <c r="B2" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="C2" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="12">
         <v>201</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="380" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
+      <c r="E2" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="380" x14ac:dyDescent="0.2">
+      <c r="A3" s="8" t="s">
         <v>22</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C3" s="11" t="s">
         <v>20</v>
@@ -10223,12 +10724,12 @@
         <v>201</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="380" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:7" ht="380" x14ac:dyDescent="0.2">
+      <c r="A4" s="8" t="s">
         <v>23</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>20</v>
@@ -10237,12 +10738,12 @@
         <v>201</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="304" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
-        <v>49</v>
+    <row r="5" spans="1:7" ht="304" x14ac:dyDescent="0.2">
+      <c r="A5" s="8" t="s">
+        <v>47</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>24</v>
@@ -10251,12 +10752,12 @@
         <v>201</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" ht="64" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="11" t="s">
         <v>28</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>29</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>24</v>
@@ -10265,12 +10766,12 @@
         <v>400</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="380" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" ht="380" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="11" t="s">
         <v>30</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>31</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>24</v>
@@ -10279,12 +10780,12 @@
         <v>400</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="380" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" ht="380" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>24</v>
@@ -10293,12 +10794,12 @@
         <v>400</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="380" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" ht="380" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>24</v>
@@ -10307,12 +10808,12 @@
         <v>400</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="304" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" ht="304" x14ac:dyDescent="0.2">
       <c r="A10" s="11" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>36</v>
+        <v>66</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>24</v>
@@ -10321,12 +10822,12 @@
         <v>400</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="304" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" ht="304" x14ac:dyDescent="0.2">
       <c r="A11" s="11" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>24</v>
@@ -10335,12 +10836,12 @@
         <v>400</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="304" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" ht="304" x14ac:dyDescent="0.2">
       <c r="A12" s="11" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>24</v>
@@ -10349,12 +10850,12 @@
         <v>400</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="304" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" ht="304" x14ac:dyDescent="0.2">
       <c r="A13" s="11" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>24</v>
@@ -10363,12 +10864,12 @@
         <v>400</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="304" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" ht="304" x14ac:dyDescent="0.2">
       <c r="A14" s="11" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>24</v>
@@ -10377,12 +10878,12 @@
         <v>400</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="304" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" ht="304" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>24</v>
@@ -10391,12 +10892,12 @@
         <v>400</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="304" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" ht="304" x14ac:dyDescent="0.2">
       <c r="A16" s="11" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C16" s="11" t="s">
         <v>24</v>
@@ -10405,63 +10906,421 @@
         <v>400</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" ht="304" x14ac:dyDescent="0.2">
       <c r="A17" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D17" s="11">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="304" x14ac:dyDescent="0.2">
+      <c r="A18" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D18" s="11">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="380" x14ac:dyDescent="0.2">
+      <c r="A19" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D19" s="11">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="380" x14ac:dyDescent="0.2">
+      <c r="A20" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D20" s="11">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="380" x14ac:dyDescent="0.2">
+      <c r="A21" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D21" s="11">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="380" x14ac:dyDescent="0.2">
+      <c r="A22" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D22" s="11">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="380" x14ac:dyDescent="0.2">
+      <c r="A23" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D23" s="11">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="380" x14ac:dyDescent="0.2">
+      <c r="A24" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24" s="11">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="382" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D25" s="11">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="382" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D26" s="11">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="382" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D27" s="11">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="380" x14ac:dyDescent="0.2">
+      <c r="A28" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="C28" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D28" s="11">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="380" x14ac:dyDescent="0.2">
+      <c r="A29" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="C29" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D29" s="11">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="380" x14ac:dyDescent="0.2">
+      <c r="A30" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="B30" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="C30" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D30" s="11">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="380" x14ac:dyDescent="0.2">
+      <c r="A31" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="B31" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="C31" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D31" s="11">
+        <v>401</v>
+      </c>
+      <c r="E31" s="11" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="380" x14ac:dyDescent="0.2">
+      <c r="A32" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="B32" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="C32" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="D32" s="11">
+        <v>404</v>
+      </c>
+      <c r="E32" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="F32" s="11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="79" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B33" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="C33" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D33" s="11">
+        <v>415</v>
+      </c>
+      <c r="E33" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="G33" s="7" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="380" x14ac:dyDescent="0.2">
+      <c r="A34" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="B34" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="C34" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D34" s="11">
+        <v>405</v>
+      </c>
+      <c r="E34" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="F34" s="11" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="380" x14ac:dyDescent="0.2">
+      <c r="A35" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="B35" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="C35" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35" s="11">
+        <v>401</v>
+      </c>
+      <c r="E35" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="F35" s="11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A36" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="C36" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D36" s="11">
+        <v>200</v>
+      </c>
+      <c r="E36" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="F36" s="11" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A37" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="C37" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="D37" s="11">
+        <v>404</v>
+      </c>
+      <c r="E37" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="F37" s="11" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A38" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="D17" s="11">
+      <c r="C38" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D38" s="11">
+        <v>405</v>
+      </c>
+      <c r="E38" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="F38" s="11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A39" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C39" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D39" s="11">
+        <v>401</v>
+      </c>
+      <c r="E39" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="F39" s="11" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="32" x14ac:dyDescent="0.2">
+      <c r="A40" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="C40" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="D40" s="11">
         <v>200</v>
       </c>
-      <c r="E17" s="11" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="80" x14ac:dyDescent="0.2">
-      <c r="A18" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="C18" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="D18" s="11">
+      <c r="F40" s="11" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="32" x14ac:dyDescent="0.2">
+      <c r="A41" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C41" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="D41" s="11">
         <v>404</v>
       </c>
-      <c r="E18" s="11" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="64" x14ac:dyDescent="0.2">
-      <c r="A19" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="C19" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="D19" s="11">
+      <c r="F41" s="11" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="32" x14ac:dyDescent="0.2">
+      <c r="A42" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="C42" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="D42" s="11">
         <v>405</v>
       </c>
-      <c r="E19" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="F19" s="11" t="s">
+      <c r="F42" s="11" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="64" x14ac:dyDescent="0.2">
-      <c r="A20" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="C20" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="D20" s="11">
+    <row r="43" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A43" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C43" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="D43" s="11">
         <v>401</v>
       </c>
-      <c r="E20" s="11" t="s">
-        <v>57</v>
+      <c r="F43" s="11" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update User module test data
</commit_message>
<xml_diff>
--- a/src/test/resources/Team01_RestAssured_Rebels_TestDataSheet.xlsx
+++ b/src/test/resources/Team01_RestAssured_Rebels_TestDataSheet.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="88">
   <si>
     <t xml:space="preserve">ScenarioName</t>
   </si>
@@ -41,6 +41,9 @@
   </si>
   <si>
     <t xml:space="preserve">Valid credential</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"userLoginEmailId":"Team01@gmail.com","password":"Team01@sep26"}</t>
   </si>
   <si>
     <t xml:space="preserve">Invalid method</t>
@@ -381,7 +384,7 @@
     <t xml:space="preserve">Get_All_Users_Valid</t>
   </si>
   <si>
-    <t xml:space="preserve">users</t>
+    <t xml:space="preserve">/users</t>
   </si>
   <si>
     <t xml:space="preserve">Get_All_Users_Invalid_Endpoint</t>
@@ -395,6 +398,78 @@
   <si>
     <t xml:space="preserve">GetAllUsers_Without_Authorization</t>
   </si>
+  <si>
+    <t xml:space="preserve">Get_Active_Inactive_User_Count_All</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[
+  {
+    "status": "Active",
+    "count": 369
+  }
+]
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">users/byStatus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Get_Active_Inactive_User_Count_R01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+  {
+    "status": "Active",
+    "count": 21
+  }
+]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Get_Active_Inactive_User_Count_R02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[
+  {
+    "status": "Active",
+    "count": 195
+  }
+]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Get_Active_Inactive_User_Count_R03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[
+  {
+    "status": "Active",
+    "count": 157
+  }
+]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Get_Active_Inactive_User_Count_Invalid_RoleID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{
+  "message": "RoleID R04 not found",
+  "success": false
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Get_Active_Inactive_User_Count_Invalid_Endpoint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">users/byStatu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Get_Active_Inactive_User_Count_Invalid_Method</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Get_Active_Inactive_User_Count_Without_Authorization</t>
+  </si>
 </sst>
 </file>
 
@@ -403,7 +478,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -439,12 +514,6 @@
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
     </font>
     <font>
       <u val="single"/>
@@ -517,7 +586,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -530,8 +599,8 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -542,23 +611,19 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -570,7 +635,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -578,32 +643,16 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -634,37 +683,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546a"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="e7e6e6"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472c4"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ed7d31"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a5a5a5"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="ffc000"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5b9bd5"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70ad47"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563c1"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954f72"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office 2013 - 2022">
@@ -837,7 +886,9 @@
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="3"/>
+      <c r="B2" s="3" t="s">
+        <v>6</v>
+      </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2" t="n">
         <v>200</v>
@@ -848,7 +899,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -861,7 +912,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -874,7 +925,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="2"/>
@@ -887,7 +938,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -898,12 +949,12 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="46.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="3" t="s">
         <v>11</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2" t="n">
@@ -913,12 +964,12 @@
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
     </row>
-    <row r="8" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="46.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2" t="n">
@@ -928,12 +979,12 @@
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" customFormat="false" ht="55.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="57.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="3" t="s">
         <v>15</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>16</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="2" t="n">
@@ -943,12 +994,12 @@
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
     </row>
-    <row r="10" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="3" t="s">
+    <row r="10" customFormat="false" ht="46.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="s">
         <v>17</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>18</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2" t="n">
@@ -958,12 +1009,12 @@
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
     </row>
-    <row r="11" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" s="3" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
         <v>19</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>20</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="2" t="n">
@@ -973,12 +1024,12 @@
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
     </row>
-    <row r="12" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" s="3" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
         <v>21</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="2" t="n">
@@ -988,12 +1039,12 @@
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
     </row>
-    <row r="13" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" s="9" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
         <v>23</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>24</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="2" t="n">
@@ -1003,12 +1054,12 @@
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
     </row>
-    <row r="14" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="B14" s="3" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="7" t="s">
         <v>25</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="2" t="n">
@@ -1018,12 +1069,12 @@
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
     </row>
-    <row r="15" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="B15" s="9" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="s">
         <v>27</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>28</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="2" t="n">
@@ -1033,12 +1084,12 @@
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
     </row>
-    <row r="16" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="B16" s="9" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="s">
         <v>29</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>30</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="2" t="n">
@@ -1049,8 +1100,8 @@
       <c r="G16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8" t="s">
-        <v>30</v>
+      <c r="A17" s="7" t="s">
+        <v>31</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -1063,7 +1114,7 @@
     </row>
     <row r="18" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2"/>
-      <c r="B18" s="8"/>
+      <c r="B18" s="7"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
@@ -1153,7 +1204,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2"/>
-      <c r="B28" s="3"/>
+      <c r="B28" s="6"/>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
@@ -1171,7 +1222,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2"/>
-      <c r="B30" s="3"/>
+      <c r="B30" s="6"/>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
@@ -1199,7 +1250,7 @@
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
-      <c r="C33" s="10"/>
+      <c r="C33" s="9"/>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
       <c r="F33" s="2"/>
@@ -9946,12 +9997,12 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B11" r:id="rId1" display="pasha.12@gmail.com"/>
-    <hyperlink ref="B12" r:id="rId2" display="Team01@gmail.com"/>
-    <hyperlink ref="B13" r:id="rId3" display="Team01@gmail.com"/>
-    <hyperlink ref="B14" r:id="rId4" display="Team01@gmail.com"/>
-    <hyperlink ref="B15" r:id="rId5" display="Team01@gmail.com"/>
-    <hyperlink ref="B16" r:id="rId6" display="inactive@gmail.com"/>
+    <hyperlink ref="B11" r:id="rId1" display="{&#10;&quot;userLoginEmailId&quot;:&quot;pasha.12@gmail.com&quot;,&#10;&quot;password&quot;:&quot;adm123&quot;&#10;}"/>
+    <hyperlink ref="B12" r:id="rId2" display="{&#10;&quot;userLoginEmailId&quot;:&quot;Team01@gmail.com&quot;,&#10;&quot;password&quot;:&quot; &quot;&#10;}"/>
+    <hyperlink ref="B13" r:id="rId3" display="{&#10;&quot;userLoginEmailId&quot;:&quot;Team01@gmail.com&quot;,&#10;&quot;password&quot;:&quot;Abc@1234$&quot;&#10;}"/>
+    <hyperlink ref="B14" r:id="rId4" display="{&#10;&quot;userLoginEmailId&quot;:&quot;Team01@gmail.com&quot;,&#10;&quot;password&quot;:&quot;adm 123&quot;&#10;}"/>
+    <hyperlink ref="B15" r:id="rId5" display="{&#10;&quot;userLoginEmailId&quot;:&quot;Team01@gmail.com&quot;,&#10;&quot;password&quot;:null&#10;}"/>
+    <hyperlink ref="B16" r:id="rId6" display="{&#10;&quot;userLoginEmailId&quot;:&quot;inactive@gmail.com&quot;,&#10;&quot;password&quot;:&quot;inactive123&quot;&#10;}"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -9971,149 +10022,148 @@
   <dimension ref="A1:M8"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="11" width="36.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="11" width="33.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="11" width="23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="11" width="19.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="11" width="14.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="36.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="10" width="33.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="10" width="23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="10" width="19.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="10" width="14.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-    </row>
-    <row r="2" customFormat="false" ht="73.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="B2" s="13" t="s">
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
+    </row>
+    <row r="2" customFormat="false" ht="75.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="B2" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="D2" s="11" t="n">
+      <c r="C2" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2" s="10" t="n">
         <v>201</v>
       </c>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
-    </row>
-    <row r="3" customFormat="false" ht="73.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="14" t="s">
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="11"/>
+      <c r="J2" s="11"/>
+      <c r="K2" s="11"/>
+      <c r="L2" s="11"/>
+      <c r="M2" s="11"/>
+    </row>
+    <row r="3" customFormat="false" ht="75.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D3" s="16" t="n">
+      <c r="D3" s="15" t="n">
         <v>201</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="73.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="B4" s="13" t="s">
+    <row r="4" customFormat="false" ht="75.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D4" s="16" t="n">
+      <c r="B4" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" s="15" t="n">
         <v>201</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="83.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="B5" s="17" t="s">
+    <row r="5" customFormat="false" ht="86.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D5" s="16" t="n">
+      <c r="B5" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" s="15" t="n">
         <v>201</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="73.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="B6" s="17" t="s">
+    <row r="6" customFormat="false" ht="75.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="C6" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D6" s="16" t="n">
+      <c r="B6" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="15" t="n">
         <v>400</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="E6" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="75.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="16" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="73.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="B7" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="C7" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="D7" s="21" t="n">
+      <c r="C7" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" s="15" t="n">
         <v>401</v>
       </c>
-      <c r="E7" s="0"/>
-    </row>
-    <row r="8" customFormat="false" ht="73.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="B8" s="19" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="75.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="C8" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="D8" s="21" t="n">
+      <c r="B8" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" s="15" t="n">
         <v>400</v>
       </c>
-      <c r="E8" s="18" t="s">
-        <v>46</v>
+      <c r="E8" s="13" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -10135,118 +10185,118 @@
   <dimension ref="A1:Z3"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="11" width="8.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="11" width="12.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="27.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="10" width="8.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="10" width="12.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="10" width="27.03"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="E1" s="12" t="s">
+      <c r="D1" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="E1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
-      <c r="O1" s="12"/>
-      <c r="P1" s="12"/>
-      <c r="Q1" s="12"/>
-      <c r="R1" s="12"/>
-      <c r="S1" s="12"/>
-      <c r="T1" s="12"/>
-      <c r="U1" s="12"/>
-      <c r="V1" s="12"/>
-      <c r="W1" s="12"/>
-      <c r="X1" s="12"/>
-      <c r="Y1" s="12"/>
-      <c r="Z1" s="12"/>
-    </row>
-    <row r="2" customFormat="false" ht="142.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="B2" s="22" t="s">
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
+      <c r="N1" s="11"/>
+      <c r="O1" s="11"/>
+      <c r="P1" s="11"/>
+      <c r="Q1" s="11"/>
+      <c r="R1" s="11"/>
+      <c r="S1" s="11"/>
+      <c r="T1" s="11"/>
+      <c r="U1" s="11"/>
+      <c r="V1" s="11"/>
+      <c r="W1" s="11"/>
+      <c r="X1" s="11"/>
+      <c r="Y1" s="11"/>
+      <c r="Z1" s="11"/>
+    </row>
+    <row r="2" customFormat="false" ht="147.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="B2" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="C2" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="E2" s="12" t="n">
+      <c r="D2" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="E2" s="11" t="n">
         <v>201</v>
       </c>
-      <c r="F2" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
-      <c r="N2" s="12"/>
-      <c r="O2" s="12"/>
-      <c r="P2" s="12"/>
-      <c r="Q2" s="12"/>
-      <c r="R2" s="12"/>
-      <c r="S2" s="12"/>
-      <c r="T2" s="12"/>
-      <c r="U2" s="12"/>
-      <c r="V2" s="12"/>
-      <c r="W2" s="12"/>
-      <c r="X2" s="12"/>
-      <c r="Y2" s="12"/>
-      <c r="Z2" s="12"/>
+      <c r="F2" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="11"/>
+      <c r="J2" s="11"/>
+      <c r="K2" s="11"/>
+      <c r="L2" s="11"/>
+      <c r="M2" s="11"/>
+      <c r="N2" s="11"/>
+      <c r="O2" s="11"/>
+      <c r="P2" s="11"/>
+      <c r="Q2" s="11"/>
+      <c r="R2" s="11"/>
+      <c r="S2" s="11"/>
+      <c r="T2" s="11"/>
+      <c r="U2" s="11"/>
+      <c r="V2" s="11"/>
+      <c r="W2" s="11"/>
+      <c r="X2" s="11"/>
+      <c r="Y2" s="11"/>
+      <c r="Z2" s="11"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="12"/>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
-      <c r="L3" s="12"/>
-      <c r="M3" s="12"/>
-      <c r="N3" s="12"/>
-      <c r="O3" s="12"/>
-      <c r="P3" s="12"/>
-      <c r="Q3" s="12"/>
-      <c r="R3" s="12"/>
-      <c r="S3" s="12"/>
-      <c r="T3" s="12"/>
-      <c r="U3" s="12"/>
-      <c r="V3" s="12"/>
-      <c r="W3" s="12"/>
-      <c r="X3" s="12"/>
-      <c r="Y3" s="12"/>
-      <c r="Z3" s="12"/>
+      <c r="A3" s="11"/>
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="11"/>
+      <c r="K3" s="11"/>
+      <c r="L3" s="11"/>
+      <c r="M3" s="11"/>
+      <c r="N3" s="11"/>
+      <c r="O3" s="11"/>
+      <c r="P3" s="11"/>
+      <c r="Q3" s="11"/>
+      <c r="R3" s="11"/>
+      <c r="S3" s="11"/>
+      <c r="T3" s="11"/>
+      <c r="U3" s="11"/>
+      <c r="V3" s="11"/>
+      <c r="W3" s="11"/>
+      <c r="X3" s="11"/>
+      <c r="Y3" s="11"/>
+      <c r="Z3" s="11"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -10264,139 +10314,257 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="23" width="8.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="23" width="61.16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="23" width="15.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="23" width="15.82"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="5" style="23" width="8.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="18" width="31.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="18" width="61.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="18" width="15.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="18" width="15.82"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="5" style="18" width="8.83"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="22.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="22" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22" t="s">
+      <c r="B1" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="22" t="s">
-        <v>53</v>
-      </c>
-      <c r="D1" s="22" t="s">
+      <c r="C1" s="17" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="261.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="22" t="s">
+      <c r="D1" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="B2" s="22" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="270.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="C2" s="22" t="s">
+      <c r="B2" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="D2" s="22" t="n">
+      <c r="C2" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2" s="17" t="n">
         <v>201</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="272.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="22" t="s">
+    <row r="3" customFormat="false" ht="282" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="B3" s="23" t="s">
-        <v>59</v>
-      </c>
-      <c r="C3" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="D3" s="23" t="n">
+      <c r="D3" s="18" t="n">
         <v>201</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="261.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="22" t="s">
-        <v>60</v>
-      </c>
-      <c r="B4" s="23" t="s">
+    <row r="4" customFormat="false" ht="270.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="C4" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="D4" s="23" t="n">
+      <c r="B4" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="D4" s="18" t="n">
         <v>201</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="207.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
-        <v>62</v>
-      </c>
-      <c r="B5" s="23" t="s">
+    <row r="5" customFormat="false" ht="214.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="B5" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="D5" s="23" t="n">
+      <c r="C5" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="D5" s="18" t="n">
         <v>201</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="22.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="B6" s="10"/>
+      <c r="C6" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="D6" s="10" t="n">
         <v>200</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="D7" s="7" t="n">
+      <c r="D8" s="10" t="n">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="D9" s="10" t="n">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="79.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>200</v>
+      </c>
+      <c r="E10" s="18" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="68.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="D11" s="10" t="n">
+        <v>200</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="68.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="D12" s="10" t="n">
+        <v>200</v>
+      </c>
+      <c r="E12" s="18" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="68.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="D13" s="10" t="n">
+        <v>200</v>
+      </c>
+      <c r="E13" s="18" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="46.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="D14" s="18" t="n">
         <v>404</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="D8" s="7" t="n">
+      <c r="E14" s="18" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="18" t="s">
+        <v>84</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="D15" s="18" t="n">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="D16" s="18" t="n">
         <v>405</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="D9" s="7" t="n">
+      <c r="E16" s="18" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="18" t="s">
+        <v>87</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="D17" s="18" t="n">
         <v>401</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
+      <c r="E17" s="18" t="s">
+        <v>75</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Add User Count API test scenarios
</commit_message>
<xml_diff>
--- a/src/test/resources/Team01_RestAssured_Rebels_TestDataSheet.xlsx
+++ b/src/test/resources/Team01_RestAssured_Rebels_TestDataSheet.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="87">
   <si>
     <t xml:space="preserve">ScenarioName</t>
   </si>
@@ -381,7 +381,7 @@
     <t xml:space="preserve">Get_All_Users_Valid</t>
   </si>
   <si>
-    <t xml:space="preserve">users</t>
+    <t xml:space="preserve">/users</t>
   </si>
   <si>
     <t xml:space="preserve">Get_All_Users_Invalid_Endpoint</t>
@@ -395,6 +395,78 @@
   <si>
     <t xml:space="preserve">GetAllUsers_Without_Authorization</t>
   </si>
+  <si>
+    <t xml:space="preserve">Get_Active_Inactive_User_Count_All</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[
+  {
+    "status": "Active",
+    "count": 369
+  }
+]
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">users/byStatus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Get_Active_Inactive_User_Count_R01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+  {
+    "status": "Active",
+    "count": 21
+  }
+]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Get_Active_Inactive_User_Count_R02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[
+  {
+    "status": "Active",
+    "count": 195
+  }
+]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Get_Active_Inactive_User_Count_R03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[
+  {
+    "status": "Active",
+    "count": 157
+  }
+]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Get_Active_Inactive_User_Count_Invalid_RoleID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{
+  "message": "RoleID R04 not found",
+  "success": false
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Get_Active_Inactive_User_Count_Invalid_Endpoint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">users/byStatu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Get_Active_Inactive_User_Count_Invalid_Method</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Get_Active_Inactive_User_Count_Without_Authorization</t>
+  </si>
 </sst>
 </file>
 
@@ -403,7 +475,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -439,12 +511,6 @@
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
     </font>
     <font>
       <u val="single"/>
@@ -517,7 +583,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="18">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -530,10 +596,6 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -542,23 +604,19 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -570,7 +628,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -578,32 +636,16 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -634,37 +676,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546a"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="e7e6e6"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472c4"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ed7d31"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a5a5a5"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="ffc000"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5b9bd5"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70ad47"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563c1"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954f72"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office 2013 - 2022">
@@ -847,7 +889,7 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="2"/>
@@ -860,7 +902,7 @@
       <c r="G3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="2"/>
@@ -873,12 +915,12 @@
       <c r="G4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="5"/>
+      <c r="B5" s="4"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="3" t="n">
         <v>415</v>
       </c>
       <c r="E5" s="2"/>
@@ -886,23 +928,23 @@
       <c r="G5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="3" t="n">
         <v>401</v>
       </c>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+    <row r="7" customFormat="false" ht="46.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="5" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="2"/>
@@ -913,11 +955,11 @@
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
     </row>
-    <row r="8" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+    <row r="8" customFormat="false" ht="46.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C8" s="2"/>
@@ -928,11 +970,11 @@
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" customFormat="false" ht="55.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+    <row r="9" customFormat="false" ht="57.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="5" t="s">
         <v>15</v>
       </c>
       <c r="C9" s="2"/>
@@ -943,11 +985,11 @@
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
     </row>
-    <row r="10" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="46.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="5" t="s">
         <v>17</v>
       </c>
       <c r="C10" s="2"/>
@@ -958,11 +1000,11 @@
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
     </row>
-    <row r="11" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="5" t="s">
         <v>19</v>
       </c>
       <c r="C11" s="2"/>
@@ -973,11 +1015,11 @@
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
     </row>
-    <row r="12" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="5" t="s">
         <v>21</v>
       </c>
       <c r="C12" s="2"/>
@@ -988,11 +1030,11 @@
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
     </row>
-    <row r="13" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="7" t="s">
         <v>23</v>
       </c>
       <c r="C13" s="2"/>
@@ -1003,11 +1045,11 @@
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
     </row>
-    <row r="14" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="5" t="s">
         <v>25</v>
       </c>
       <c r="C14" s="2"/>
@@ -1018,11 +1060,11 @@
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
     </row>
-    <row r="15" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="7" t="s">
         <v>27</v>
       </c>
       <c r="C15" s="2"/>
@@ -1033,11 +1075,11 @@
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
     </row>
-    <row r="16" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="7" t="s">
         <v>29</v>
       </c>
       <c r="C16" s="2"/>
@@ -1049,7 +1091,7 @@
       <c r="G16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="6" t="s">
         <v>30</v>
       </c>
       <c r="B17" s="2"/>
@@ -1063,7 +1105,7 @@
     </row>
     <row r="18" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2"/>
-      <c r="B18" s="8"/>
+      <c r="B18" s="6"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
@@ -1153,7 +1195,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2"/>
-      <c r="B28" s="3"/>
+      <c r="B28" s="5"/>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
@@ -1171,7 +1213,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2"/>
-      <c r="B30" s="3"/>
+      <c r="B30" s="5"/>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
@@ -1199,7 +1241,7 @@
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
-      <c r="C33" s="10"/>
+      <c r="C33" s="8"/>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
       <c r="F33" s="2"/>
@@ -9946,12 +9988,12 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B11" r:id="rId1" display="pasha.12@gmail.com"/>
-    <hyperlink ref="B12" r:id="rId2" display="Team01@gmail.com"/>
-    <hyperlink ref="B13" r:id="rId3" display="Team01@gmail.com"/>
-    <hyperlink ref="B14" r:id="rId4" display="Team01@gmail.com"/>
-    <hyperlink ref="B15" r:id="rId5" display="Team01@gmail.com"/>
-    <hyperlink ref="B16" r:id="rId6" display="inactive@gmail.com"/>
+    <hyperlink ref="B11" r:id="rId1" display="{&#10;&quot;userLoginEmailId&quot;:&quot;pasha.12@gmail.com&quot;,&#10;&quot;password&quot;:&quot;adm123&quot;&#10;}"/>
+    <hyperlink ref="B12" r:id="rId2" display="{&#10;&quot;userLoginEmailId&quot;:&quot;Team01@gmail.com&quot;,&#10;&quot;password&quot;:&quot; &quot;&#10;}"/>
+    <hyperlink ref="B13" r:id="rId3" display="{&#10;&quot;userLoginEmailId&quot;:&quot;Team01@gmail.com&quot;,&#10;&quot;password&quot;:&quot;Abc@1234$&quot;&#10;}"/>
+    <hyperlink ref="B14" r:id="rId4" display="{&#10;&quot;userLoginEmailId&quot;:&quot;Team01@gmail.com&quot;,&#10;&quot;password&quot;:&quot;adm 123&quot;&#10;}"/>
+    <hyperlink ref="B15" r:id="rId5" display="{&#10;&quot;userLoginEmailId&quot;:&quot;Team01@gmail.com&quot;,&#10;&quot;password&quot;:null&#10;}"/>
+    <hyperlink ref="B16" r:id="rId6" display="{&#10;&quot;userLoginEmailId&quot;:&quot;inactive@gmail.com&quot;,&#10;&quot;password&quot;:&quot;inactive123&quot;&#10;}"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -9971,148 +10013,147 @@
   <dimension ref="A1:M8"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="11" width="36.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="11" width="33.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="11" width="23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="11" width="19.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="11" width="14.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="9" width="36.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="9" width="33.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="9" width="23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="9" width="19.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="9" width="14.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-    </row>
-    <row r="2" customFormat="false" ht="73.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="11" t="s">
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+    </row>
+    <row r="2" customFormat="false" ht="75.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="D2" s="11" t="n">
+      <c r="D2" s="9" t="n">
         <v>201</v>
       </c>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
-    </row>
-    <row r="3" customFormat="false" ht="73.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="14" t="s">
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="10"/>
+      <c r="K2" s="10"/>
+      <c r="L2" s="10"/>
+      <c r="M2" s="10"/>
+    </row>
+    <row r="3" customFormat="false" ht="75.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="D3" s="16" t="n">
+      <c r="D3" s="14" t="n">
         <v>201</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="73.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="14" t="s">
+    <row r="4" customFormat="false" ht="75.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="D4" s="16" t="n">
+      <c r="D4" s="14" t="n">
         <v>201</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="83.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14" t="s">
+    <row r="5" customFormat="false" ht="86.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="16" t="n">
+      <c r="D5" s="14" t="n">
         <v>201</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="73.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="14" t="s">
+    <row r="6" customFormat="false" ht="75.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="16" t="n">
+      <c r="D6" s="14" t="n">
         <v>400</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="E6" s="15" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="73.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
+    <row r="7" customFormat="false" ht="75.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="C7" s="20" t="s">
+      <c r="C7" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="D7" s="21" t="n">
+      <c r="D7" s="14" t="n">
         <v>401</v>
       </c>
-      <c r="E7" s="0"/>
-    </row>
-    <row r="8" customFormat="false" ht="73.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="75.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="C8" s="20" t="s">
+      <c r="C8" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="21" t="n">
+      <c r="D8" s="14" t="n">
         <v>400</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="E8" s="12" t="s">
         <v>46</v>
       </c>
     </row>
@@ -10135,118 +10176,118 @@
   <dimension ref="A1:Z3"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="11" width="8.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="11" width="12.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="27.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="9" width="8.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="9" width="12.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="9" width="27.03"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
-      <c r="O1" s="12"/>
-      <c r="P1" s="12"/>
-      <c r="Q1" s="12"/>
-      <c r="R1" s="12"/>
-      <c r="S1" s="12"/>
-      <c r="T1" s="12"/>
-      <c r="U1" s="12"/>
-      <c r="V1" s="12"/>
-      <c r="W1" s="12"/>
-      <c r="X1" s="12"/>
-      <c r="Y1" s="12"/>
-      <c r="Z1" s="12"/>
-    </row>
-    <row r="2" customFormat="false" ht="142.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="12" t="s">
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="10"/>
+      <c r="P1" s="10"/>
+      <c r="Q1" s="10"/>
+      <c r="R1" s="10"/>
+      <c r="S1" s="10"/>
+      <c r="T1" s="10"/>
+      <c r="U1" s="10"/>
+      <c r="V1" s="10"/>
+      <c r="W1" s="10"/>
+      <c r="X1" s="10"/>
+      <c r="Y1" s="10"/>
+      <c r="Z1" s="10"/>
+    </row>
+    <row r="2" customFormat="false" ht="147.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="E2" s="12" t="n">
+      <c r="E2" s="10" t="n">
         <v>201</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="F2" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
-      <c r="N2" s="12"/>
-      <c r="O2" s="12"/>
-      <c r="P2" s="12"/>
-      <c r="Q2" s="12"/>
-      <c r="R2" s="12"/>
-      <c r="S2" s="12"/>
-      <c r="T2" s="12"/>
-      <c r="U2" s="12"/>
-      <c r="V2" s="12"/>
-      <c r="W2" s="12"/>
-      <c r="X2" s="12"/>
-      <c r="Y2" s="12"/>
-      <c r="Z2" s="12"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="10"/>
+      <c r="K2" s="10"/>
+      <c r="L2" s="10"/>
+      <c r="M2" s="10"/>
+      <c r="N2" s="10"/>
+      <c r="O2" s="10"/>
+      <c r="P2" s="10"/>
+      <c r="Q2" s="10"/>
+      <c r="R2" s="10"/>
+      <c r="S2" s="10"/>
+      <c r="T2" s="10"/>
+      <c r="U2" s="10"/>
+      <c r="V2" s="10"/>
+      <c r="W2" s="10"/>
+      <c r="X2" s="10"/>
+      <c r="Y2" s="10"/>
+      <c r="Z2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="12"/>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
-      <c r="L3" s="12"/>
-      <c r="M3" s="12"/>
-      <c r="N3" s="12"/>
-      <c r="O3" s="12"/>
-      <c r="P3" s="12"/>
-      <c r="Q3" s="12"/>
-      <c r="R3" s="12"/>
-      <c r="S3" s="12"/>
-      <c r="T3" s="12"/>
-      <c r="U3" s="12"/>
-      <c r="V3" s="12"/>
-      <c r="W3" s="12"/>
-      <c r="X3" s="12"/>
-      <c r="Y3" s="12"/>
-      <c r="Z3" s="12"/>
+      <c r="A3" s="10"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="10"/>
+      <c r="M3" s="10"/>
+      <c r="N3" s="10"/>
+      <c r="O3" s="10"/>
+      <c r="P3" s="10"/>
+      <c r="Q3" s="10"/>
+      <c r="R3" s="10"/>
+      <c r="S3" s="10"/>
+      <c r="T3" s="10"/>
+      <c r="U3" s="10"/>
+      <c r="V3" s="10"/>
+      <c r="W3" s="10"/>
+      <c r="X3" s="10"/>
+      <c r="Y3" s="10"/>
+      <c r="Z3" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -10264,139 +10305,257 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="23" width="8.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="23" width="61.16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="23" width="15.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="23" width="15.82"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="5" style="23" width="8.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="17" width="31.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="17" width="61.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="17" width="15.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="17" width="15.82"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="5" style="17" width="8.83"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="22.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="22" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22" t="s">
+      <c r="B1" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="22" t="s">
+      <c r="C1" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="D1" s="22" t="s">
+      <c r="D1" s="16" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="261.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="22" t="s">
+    <row r="2" customFormat="false" ht="270.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="C2" s="22" t="s">
+      <c r="C2" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="D2" s="22" t="n">
+      <c r="D2" s="16" t="n">
         <v>201</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="272.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="22" t="s">
+    <row r="3" customFormat="false" ht="282" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="B3" s="23" t="s">
+      <c r="B3" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="C3" s="23" t="s">
+      <c r="C3" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="D3" s="23" t="n">
+      <c r="D3" s="17" t="n">
         <v>201</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="261.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="22" t="s">
+    <row r="4" customFormat="false" ht="270.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="C4" s="23" t="s">
+      <c r="C4" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="D4" s="23" t="n">
+      <c r="D4" s="17" t="n">
         <v>201</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="207.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
+    <row r="5" customFormat="false" ht="214.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="B5" s="23" t="s">
+      <c r="B5" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="C5" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="D5" s="23" t="n">
+      <c r="D5" s="17" t="n">
         <v>201</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="22.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7" t="s">
+      <c r="B6" s="9"/>
+      <c r="C6" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="9" t="n">
         <v>200</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7" t="s">
+      <c r="B7" s="9"/>
+      <c r="C7" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="9" t="n">
         <v>404</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7" t="s">
+      <c r="B8" s="9"/>
+      <c r="C8" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="9" t="n">
         <v>405</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7" t="s">
+      <c r="B9" s="9"/>
+      <c r="C9" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="9" t="n">
         <v>401</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
+    <row r="10" customFormat="false" ht="79.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>200</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="68.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>200</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="68.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>200</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="68.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>200</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="46.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="B14" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D14" s="17" t="n">
+        <v>404</v>
+      </c>
+      <c r="E14" s="17" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="D15" s="17" t="n">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D16" s="17" t="n">
+        <v>405</v>
+      </c>
+      <c r="E16" s="17" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D17" s="17" t="n">
+        <v>401</v>
+      </c>
+      <c r="E17" s="17" t="s">
+        <v>74</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>